<commit_message>
tema 6 inicialmente preparado
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/matricula_asistencia_notas_Caucasia_2026-2.xlsx
+++ b/9_asistencia_evaluacion/matricula_asistencia_notas_Caucasia_2026-2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F23D9A-971A-4006-9C7E-7C5292FE94A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256F4971-926A-4A11-89AD-2199E675AFD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="116">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -1088,6 +1088,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1118,15 +1196,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1170,75 +1239,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1721,7 +1721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.26953125" bestFit="1" customWidth="1"/>
@@ -2468,227 +2468,217 @@
     </row>
     <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
-        <v>32</v>
-      </c>
-      <c r="B35" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C35" s="43" t="s">
+      <c r="C35" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="43">
+      <c r="D35" s="15">
         <v>1038648764</v>
       </c>
       <c r="E35" s="14"/>
-      <c r="F35" s="43">
+      <c r="F35" s="14">
         <v>3132068325</v>
       </c>
-      <c r="G35" s="43" t="s">
+      <c r="G35" s="45" t="s">
         <v>68</v>
       </c>
       <c r="H35" s="14"/>
     </row>
     <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
-        <v>33</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D36" s="15">
-        <v>1038648764</v>
+        <v>34</v>
+      </c>
+      <c r="B36" s="43" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" s="43">
+        <v>1038118107</v>
       </c>
       <c r="E36" s="14"/>
-      <c r="F36" s="14">
-        <v>3132068325</v>
-      </c>
-      <c r="G36" s="45" t="s">
-        <v>68</v>
+      <c r="F36" s="43">
+        <v>3125629643</v>
+      </c>
+      <c r="G36" s="43" t="s">
+        <v>83</v>
       </c>
       <c r="H36" s="14"/>
     </row>
     <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B37" s="43" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C37" s="43" t="s">
         <v>65</v>
       </c>
       <c r="D37" s="43">
-        <v>1038118107</v>
+        <v>1020303245</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="43">
-        <v>3125629643</v>
+        <v>3132893979</v>
       </c>
       <c r="G37" s="43" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="H37" s="14"/>
     </row>
     <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B38" s="43" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C38" s="43" t="s">
         <v>65</v>
       </c>
       <c r="D38" s="43">
-        <v>1020303245</v>
+        <v>1045143166</v>
       </c>
       <c r="E38" s="14"/>
       <c r="F38" s="43">
-        <v>3132893979</v>
+        <v>3145252170</v>
       </c>
       <c r="G38" s="43" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H38" s="14"/>
     </row>
     <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B39" s="43" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="C39" s="43" t="s">
         <v>65</v>
       </c>
       <c r="D39" s="43">
-        <v>1045143166</v>
+        <v>1038116526</v>
       </c>
       <c r="E39" s="14"/>
       <c r="F39" s="43">
-        <v>3145252170</v>
-      </c>
-      <c r="G39" s="43" t="s">
-        <v>77</v>
+        <v>3332364722</v>
+      </c>
+      <c r="G39" s="46" t="s">
+        <v>111</v>
       </c>
       <c r="H39" s="14"/>
     </row>
     <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="10">
-        <v>37</v>
-      </c>
-      <c r="B40" s="43" t="s">
-        <v>32</v>
+        <v>38</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>97</v>
       </c>
       <c r="C40" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="D40" s="43">
-        <v>1038116526</v>
+      <c r="D40" s="15">
+        <v>1040502849</v>
       </c>
       <c r="E40" s="14"/>
-      <c r="F40" s="43">
-        <v>3332364722</v>
-      </c>
-      <c r="G40" s="46" t="s">
-        <v>111</v>
+      <c r="F40" s="14">
+        <v>3218908879</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>98</v>
       </c>
       <c r="H40" s="14"/>
     </row>
     <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="10">
-        <v>38</v>
-      </c>
-      <c r="B41" s="15" t="s">
-        <v>97</v>
+        <v>39</v>
+      </c>
+      <c r="B41" s="43" t="s">
+        <v>55</v>
       </c>
       <c r="C41" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="D41" s="15">
-        <v>1040502849</v>
+      <c r="D41" s="43" t="s">
+        <v>66</v>
       </c>
       <c r="E41" s="14"/>
-      <c r="F41" s="14">
-        <v>3218908879</v>
-      </c>
-      <c r="G41" s="17" t="s">
-        <v>98</v>
+      <c r="F41" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="G41" s="43" t="s">
+        <v>89</v>
       </c>
       <c r="H41" s="14"/>
     </row>
     <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="10">
-        <v>39</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="D42" s="43" t="s">
-        <v>66</v>
+        <v>40</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" s="15">
+        <v>1038125682</v>
       </c>
       <c r="E42" s="14"/>
-      <c r="F42" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="G42" s="43" t="s">
-        <v>89</v>
+      <c r="F42" s="14">
+        <v>3116434791</v>
+      </c>
+      <c r="G42" s="45" t="s">
+        <v>113</v>
       </c>
       <c r="H42" s="14"/>
     </row>
     <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>104</v>
       </c>
       <c r="D43" s="15">
-        <v>1038125682</v>
+        <v>33104650</v>
       </c>
       <c r="E43" s="14"/>
       <c r="F43" s="14">
-        <v>3116434791</v>
+        <v>31466565745</v>
       </c>
       <c r="G43" s="45" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H43" s="14"/>
     </row>
     <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="10">
-        <v>41</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C44" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D44" s="15">
-        <v>33104650</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
       <c r="E44" s="14"/>
-      <c r="F44" s="14">
-        <v>31466565745</v>
-      </c>
-      <c r="G44" s="45" t="s">
-        <v>115</v>
-      </c>
+      <c r="F44" s="14"/>
+      <c r="G44" s="17"/>
       <c r="H44" s="14"/>
     </row>
     <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
@@ -2700,7 +2690,7 @@
     </row>
     <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="10">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
@@ -2712,7 +2702,7 @@
     </row>
     <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
@@ -2724,7 +2714,7 @@
     </row>
     <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="10">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
@@ -2736,7 +2726,7 @@
     </row>
     <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="10">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
@@ -2748,7 +2738,7 @@
     </row>
     <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="10">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -2760,7 +2750,7 @@
     </row>
     <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="10">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
@@ -2772,7 +2762,7 @@
     </row>
     <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="10">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
@@ -2784,7 +2774,7 @@
     </row>
     <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="10">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B53" s="15"/>
       <c r="C53" s="15"/>
@@ -2796,7 +2786,7 @@
     </row>
     <row r="54" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="10">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
@@ -2808,7 +2798,7 @@
     </row>
     <row r="55" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="10">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
@@ -2820,7 +2810,7 @@
     </row>
     <row r="56" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="10">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
@@ -2832,7 +2822,7 @@
     </row>
     <row r="57" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -2844,7 +2834,7 @@
     </row>
     <row r="58" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="10">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
@@ -2856,7 +2846,7 @@
     </row>
     <row r="59" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="10">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
@@ -2868,7 +2858,7 @@
     </row>
     <row r="60" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="10">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
@@ -2880,7 +2870,7 @@
     </row>
     <row r="61" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="10">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
@@ -2892,7 +2882,7 @@
     </row>
     <row r="62" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="10">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
@@ -2902,21 +2892,9 @@
       <c r="G62" s="17"/>
       <c r="H62" s="14"/>
     </row>
-    <row r="63" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="10">
-        <v>60</v>
-      </c>
-      <c r="B63" s="15"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="17"/>
-      <c r="H63" s="14"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:H42">
-    <sortCondition ref="B4:B42"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B4:H41">
+    <sortCondition ref="B4:B41"/>
   </sortState>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -2928,14 +2906,14 @@
     <hyperlink ref="G13" r:id="rId2" xr:uid="{C5973669-08D4-4EDB-BC88-68C473FA1CE3}"/>
     <hyperlink ref="G32" r:id="rId3" xr:uid="{3BD91535-3D01-463C-8CCA-D89045539993}"/>
     <hyperlink ref="G24" r:id="rId4" xr:uid="{746370CC-A7A7-415A-A5E9-F6AFD8BF2B1F}"/>
-    <hyperlink ref="G36" r:id="rId5" xr:uid="{B1EF5833-1719-4014-9B02-97215BECB266}"/>
+    <hyperlink ref="G35" r:id="rId5" xr:uid="{B1EF5833-1719-4014-9B02-97215BECB266}"/>
     <hyperlink ref="G12" r:id="rId6" xr:uid="{1A57B07E-8E3A-46FF-8553-08EAA206C617}"/>
     <hyperlink ref="G27" r:id="rId7" xr:uid="{C24D9F3D-2654-4B54-990D-FC0A5F15A97D}"/>
     <hyperlink ref="G22" r:id="rId8" xr:uid="{8C70339C-1B33-4C80-BB8E-6C1DAC47D612}"/>
     <hyperlink ref="G8" r:id="rId9" xr:uid="{7410146B-0C3D-43D1-B729-BE5671A1A2B1}"/>
-    <hyperlink ref="G40" r:id="rId10" xr:uid="{A6D3AE4C-77D8-4128-87E1-5474F08EADEB}"/>
-    <hyperlink ref="G43" r:id="rId11" xr:uid="{54BDB88E-CE45-4C75-86A6-A24DF4F78D4D}"/>
-    <hyperlink ref="G44" r:id="rId12" xr:uid="{F9BDA904-CAE2-409A-A474-5CB00EEA97A8}"/>
+    <hyperlink ref="G39" r:id="rId10" xr:uid="{A6D3AE4C-77D8-4128-87E1-5474F08EADEB}"/>
+    <hyperlink ref="G42" r:id="rId11" xr:uid="{54BDB88E-CE45-4C75-86A6-A24DF4F78D4D}"/>
+    <hyperlink ref="G43" r:id="rId12" xr:uid="{F9BDA904-CAE2-409A-A474-5CB00EEA97A8}"/>
   </hyperlinks>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId13"/>
@@ -2945,7 +2923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AE65"/>
+  <dimension ref="A1:AE64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="34.54296875" bestFit="1" customWidth="1"/>
@@ -3135,7 +3113,7 @@
         <v>18</v>
       </c>
       <c r="I5" s="44">
-        <v>46258</v>
+        <v>46272</v>
       </c>
       <c r="J5" s="44">
         <v>46259</v>
@@ -3192,7 +3170,9 @@
         <f>+SUM(D6:G6)/4</f>
         <v>0</v>
       </c>
-      <c r="I6" s="38"/>
+      <c r="I6" s="38">
+        <v>1</v>
+      </c>
       <c r="J6" s="38"/>
       <c r="K6" s="38"/>
       <c r="L6" s="38"/>
@@ -3202,7 +3182,7 @@
       <c r="P6" s="38"/>
       <c r="Q6" s="37">
         <f>+SUM(I6:P6)/8</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R6" s="38"/>
       <c r="S6" s="38"/>
@@ -3242,10 +3222,12 @@
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="37">
-        <f t="shared" ref="H7:H55" si="0">+SUM(D7:G7)/4</f>
-        <v>0</v>
-      </c>
-      <c r="I7" s="38"/>
+        <f t="shared" ref="H7:H54" si="0">+SUM(D7:G7)/4</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="38">
+        <v>0</v>
+      </c>
       <c r="J7" s="38"/>
       <c r="K7" s="38"/>
       <c r="L7" s="38"/>
@@ -3254,7 +3236,7 @@
       <c r="O7" s="38"/>
       <c r="P7" s="39"/>
       <c r="Q7" s="37">
-        <f t="shared" ref="Q7:Q55" si="1">+SUM(I7:P7)/8</f>
+        <f t="shared" ref="Q7:Q54" si="1">+SUM(I7:P7)/8</f>
         <v>0</v>
       </c>
       <c r="R7" s="38"/>
@@ -3266,7 +3248,7 @@
       <c r="X7" s="39"/>
       <c r="Y7" s="38"/>
       <c r="Z7" s="37">
-        <f t="shared" ref="Z7:Z55" si="2">+SUM(R7:Y7)/8</f>
+        <f t="shared" ref="Z7:Z54" si="2">+SUM(R7:Y7)/8</f>
         <v>0</v>
       </c>
       <c r="AA7" s="40"/>
@@ -3274,7 +3256,7 @@
       <c r="AC7" s="39"/>
       <c r="AD7" s="39"/>
       <c r="AE7" s="37">
-        <f t="shared" ref="AE7:AE55" si="3">+SUM(AA7:AD7)/4</f>
+        <f t="shared" ref="AE7:AE54" si="3">+SUM(AA7:AD7)/4</f>
         <v>0</v>
       </c>
     </row>
@@ -3298,7 +3280,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I8" s="38"/>
+      <c r="I8" s="38">
+        <v>0</v>
+      </c>
       <c r="J8" s="38"/>
       <c r="K8" s="38"/>
       <c r="L8" s="38"/>
@@ -3351,7 +3335,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I9" s="38"/>
+      <c r="I9" s="38">
+        <v>0</v>
+      </c>
       <c r="J9" s="38"/>
       <c r="K9" s="38"/>
       <c r="L9" s="38"/>
@@ -3404,7 +3390,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I10" s="38"/>
+      <c r="I10" s="38">
+        <v>0</v>
+      </c>
       <c r="J10" s="38"/>
       <c r="K10" s="38"/>
       <c r="L10" s="38"/>
@@ -3457,7 +3445,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I11" s="38"/>
+      <c r="I11" s="38">
+        <v>0</v>
+      </c>
       <c r="J11" s="38"/>
       <c r="K11" s="38"/>
       <c r="L11" s="38"/>
@@ -3510,7 +3500,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I12" s="38"/>
+      <c r="I12" s="38">
+        <v>0</v>
+      </c>
       <c r="J12" s="38"/>
       <c r="K12" s="38"/>
       <c r="L12" s="38"/>
@@ -3563,7 +3555,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I13" s="38"/>
+      <c r="I13" s="38">
+        <v>1</v>
+      </c>
       <c r="J13" s="38"/>
       <c r="K13" s="38"/>
       <c r="L13" s="38"/>
@@ -3573,7 +3567,7 @@
       <c r="P13" s="39"/>
       <c r="Q13" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R13" s="38"/>
       <c r="S13" s="38"/>
@@ -3616,7 +3610,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I14" s="38"/>
+      <c r="I14" s="38">
+        <v>0</v>
+      </c>
       <c r="J14" s="38"/>
       <c r="K14" s="38"/>
       <c r="L14" s="38"/>
@@ -3669,7 +3665,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I15" s="38"/>
+      <c r="I15" s="38">
+        <v>0</v>
+      </c>
       <c r="J15" s="38"/>
       <c r="K15" s="38"/>
       <c r="L15" s="38"/>
@@ -3722,7 +3720,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I16" s="38"/>
+      <c r="I16" s="38">
+        <v>1</v>
+      </c>
       <c r="J16" s="38"/>
       <c r="K16" s="38"/>
       <c r="L16" s="38"/>
@@ -3732,7 +3732,7 @@
       <c r="P16" s="39"/>
       <c r="Q16" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R16" s="38"/>
       <c r="S16" s="38"/>
@@ -3775,7 +3775,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I17" s="38"/>
+      <c r="I17" s="38">
+        <v>0</v>
+      </c>
       <c r="J17" s="38"/>
       <c r="K17" s="38"/>
       <c r="L17" s="38"/>
@@ -3828,7 +3830,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I18" s="38"/>
+      <c r="I18" s="38">
+        <v>1</v>
+      </c>
       <c r="J18" s="38"/>
       <c r="K18" s="38"/>
       <c r="L18" s="38"/>
@@ -3838,7 +3842,7 @@
       <c r="P18" s="39"/>
       <c r="Q18" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R18" s="38"/>
       <c r="S18" s="38"/>
@@ -3881,7 +3885,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I19" s="38"/>
+      <c r="I19" s="38">
+        <v>0</v>
+      </c>
       <c r="J19" s="38"/>
       <c r="K19" s="38"/>
       <c r="L19" s="38"/>
@@ -3934,7 +3940,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I20" s="38"/>
+      <c r="I20" s="38">
+        <v>1</v>
+      </c>
       <c r="J20" s="38"/>
       <c r="K20" s="38"/>
       <c r="L20" s="38"/>
@@ -3944,7 +3952,7 @@
       <c r="P20" s="39"/>
       <c r="Q20" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R20" s="38"/>
       <c r="S20" s="38"/>
@@ -3987,7 +3995,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I21" s="38"/>
+      <c r="I21" s="38">
+        <v>1</v>
+      </c>
       <c r="J21" s="38"/>
       <c r="K21" s="38"/>
       <c r="L21" s="38"/>
@@ -3997,7 +4007,7 @@
       <c r="P21" s="39"/>
       <c r="Q21" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R21" s="38"/>
       <c r="S21" s="38"/>
@@ -4040,7 +4050,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I22" s="38"/>
+      <c r="I22" s="38">
+        <v>1</v>
+      </c>
       <c r="J22" s="38">
         <v>1</v>
       </c>
@@ -4052,7 +4064,7 @@
       <c r="P22" s="38"/>
       <c r="Q22" s="37">
         <f t="shared" si="1"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="R22" s="38"/>
       <c r="S22" s="38"/>
@@ -4095,7 +4107,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I23" s="38"/>
+      <c r="I23" s="38">
+        <v>1</v>
+      </c>
       <c r="J23" s="38"/>
       <c r="K23" s="38"/>
       <c r="L23" s="38"/>
@@ -4105,7 +4119,7 @@
       <c r="P23" s="39"/>
       <c r="Q23" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R23" s="38"/>
       <c r="S23" s="38"/>
@@ -4148,7 +4162,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I24" s="38"/>
+      <c r="I24" s="38">
+        <v>1</v>
+      </c>
       <c r="J24" s="38"/>
       <c r="K24" s="38"/>
       <c r="L24" s="38"/>
@@ -4158,7 +4174,7 @@
       <c r="P24" s="39"/>
       <c r="Q24" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R24" s="38"/>
       <c r="S24" s="38"/>
@@ -4201,7 +4217,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I25" s="38"/>
+      <c r="I25" s="38">
+        <v>0</v>
+      </c>
       <c r="J25" s="38"/>
       <c r="K25" s="38"/>
       <c r="L25" s="38"/>
@@ -4254,7 +4272,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I26" s="38"/>
+      <c r="I26" s="38">
+        <v>1</v>
+      </c>
       <c r="J26" s="38"/>
       <c r="K26" s="38"/>
       <c r="L26" s="38"/>
@@ -4264,7 +4284,7 @@
       <c r="P26" s="38"/>
       <c r="Q26" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R26" s="38"/>
       <c r="S26" s="38"/>
@@ -4307,7 +4327,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I27" s="38"/>
+      <c r="I27" s="38">
+        <v>1</v>
+      </c>
       <c r="J27" s="38"/>
       <c r="K27" s="38"/>
       <c r="L27" s="38"/>
@@ -4317,7 +4339,7 @@
       <c r="P27" s="39"/>
       <c r="Q27" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R27" s="38"/>
       <c r="S27" s="38"/>
@@ -4360,7 +4382,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I28" s="38"/>
+      <c r="I28" s="38">
+        <v>1</v>
+      </c>
       <c r="J28" s="38"/>
       <c r="K28" s="38"/>
       <c r="L28" s="38"/>
@@ -4370,7 +4394,7 @@
       <c r="P28" s="39"/>
       <c r="Q28" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R28" s="38"/>
       <c r="S28" s="38"/>
@@ -4413,7 +4437,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I29" s="38"/>
+      <c r="I29" s="38">
+        <v>1</v>
+      </c>
       <c r="J29" s="38"/>
       <c r="K29" s="38"/>
       <c r="L29" s="38"/>
@@ -4423,7 +4449,7 @@
       <c r="P29" s="39"/>
       <c r="Q29" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R29" s="38"/>
       <c r="S29" s="38"/>
@@ -4466,7 +4492,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I30" s="38"/>
+      <c r="I30" s="38">
+        <v>0</v>
+      </c>
       <c r="J30" s="38"/>
       <c r="K30" s="38"/>
       <c r="L30" s="38"/>
@@ -4519,7 +4547,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I31" s="38"/>
+      <c r="I31" s="38">
+        <v>0</v>
+      </c>
       <c r="J31" s="38"/>
       <c r="K31" s="38"/>
       <c r="L31" s="38"/>
@@ -4572,7 +4602,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I32" s="38"/>
+      <c r="I32" s="38">
+        <v>1</v>
+      </c>
       <c r="J32" s="38"/>
       <c r="K32" s="38"/>
       <c r="L32" s="38"/>
@@ -4582,7 +4614,7 @@
       <c r="P32" s="39"/>
       <c r="Q32" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R32" s="38"/>
       <c r="S32" s="38"/>
@@ -4625,7 +4657,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I33" s="38"/>
+      <c r="I33" s="38">
+        <v>0</v>
+      </c>
       <c r="J33" s="38"/>
       <c r="K33" s="38"/>
       <c r="L33" s="38"/>
@@ -4678,7 +4712,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I34" s="38"/>
+      <c r="I34" s="38">
+        <v>0</v>
+      </c>
       <c r="J34" s="38"/>
       <c r="K34" s="38"/>
       <c r="L34" s="38"/>
@@ -4731,7 +4767,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I35" s="38"/>
+      <c r="I35" s="38">
+        <v>0</v>
+      </c>
       <c r="J35" s="38"/>
       <c r="K35" s="38"/>
       <c r="L35" s="38"/>
@@ -4784,7 +4822,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I36" s="38"/>
+      <c r="I36" s="38">
+        <v>1</v>
+      </c>
       <c r="J36" s="38"/>
       <c r="K36" s="38"/>
       <c r="L36" s="38"/>
@@ -4794,7 +4834,7 @@
       <c r="P36" s="39"/>
       <c r="Q36" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R36" s="38"/>
       <c r="S36" s="38"/>
@@ -4817,9 +4857,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:31" s="19" customFormat="1" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A37" s="20">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" s="18" t="str">
         <f>+Inscritos!B35</f>
@@ -4837,17 +4877,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I37" s="38"/>
+      <c r="I37" s="38">
+        <v>1</v>
+      </c>
       <c r="J37" s="38"/>
       <c r="K37" s="38"/>
       <c r="L37" s="38"/>
       <c r="M37" s="38"/>
       <c r="N37" s="38"/>
       <c r="O37" s="38"/>
-      <c r="P37" s="38"/>
+      <c r="P37" s="39"/>
       <c r="Q37" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R37" s="38"/>
       <c r="S37" s="38"/>
@@ -4861,10 +4903,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA37" s="41"/>
-      <c r="AB37" s="42"/>
-      <c r="AC37" s="42"/>
-      <c r="AD37" s="42"/>
+      <c r="AA37" s="40"/>
+      <c r="AB37" s="39"/>
+      <c r="AC37" s="39"/>
+      <c r="AD37" s="39"/>
       <c r="AE37" s="37">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -4872,15 +4914,15 @@
     </row>
     <row r="38" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A38" s="20">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B38" s="18" t="str">
         <f>+Inscritos!B36</f>
-        <v>Sara Paulina Cardona Almanza</v>
+        <v>Sheyla Ramirez Guerra</v>
       </c>
       <c r="C38" s="21">
         <f>+Inscritos!D36</f>
-        <v>1038648764</v>
+        <v>1038118107</v>
       </c>
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
@@ -4890,7 +4932,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I38" s="38"/>
+      <c r="I38" s="38">
+        <v>1</v>
+      </c>
       <c r="J38" s="38"/>
       <c r="K38" s="38"/>
       <c r="L38" s="38"/>
@@ -4900,7 +4944,7 @@
       <c r="P38" s="39"/>
       <c r="Q38" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R38" s="38"/>
       <c r="S38" s="38"/>
@@ -4925,15 +4969,15 @@
     </row>
     <row r="39" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A39" s="20">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B39" s="18" t="str">
         <f>+Inscritos!B37</f>
-        <v>Sheyla Ramirez Guerra</v>
+        <v>Susana Tobon Ortega</v>
       </c>
       <c r="C39" s="21">
         <f>+Inscritos!D37</f>
-        <v>1038118107</v>
+        <v>1020303245</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
@@ -4943,7 +4987,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I39" s="38"/>
+      <c r="I39" s="38">
+        <v>0</v>
+      </c>
       <c r="J39" s="38"/>
       <c r="K39" s="38"/>
       <c r="L39" s="38"/>
@@ -4978,15 +5024,15 @@
     </row>
     <row r="40" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A40" s="20">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B40" s="18" t="str">
         <f>+Inscritos!B38</f>
-        <v>Susana Tobon Ortega</v>
+        <v xml:space="preserve">Valerin Fernanda  Pérez Mejía </v>
       </c>
       <c r="C40" s="21">
         <f>+Inscritos!D38</f>
-        <v>1020303245</v>
+        <v>1045143166</v>
       </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
@@ -4996,17 +5042,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I40" s="38"/>
+      <c r="I40" s="38">
+        <v>1</v>
+      </c>
       <c r="J40" s="38"/>
       <c r="K40" s="38"/>
       <c r="L40" s="38"/>
       <c r="M40" s="38"/>
       <c r="N40" s="38"/>
       <c r="O40" s="38"/>
-      <c r="P40" s="39"/>
+      <c r="P40" s="38"/>
       <c r="Q40" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R40" s="38"/>
       <c r="S40" s="38"/>
@@ -5031,15 +5079,15 @@
     </row>
     <row r="41" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A41" s="20">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B41" s="18" t="str">
         <f>+Inscritos!B39</f>
-        <v xml:space="preserve">Valerin Fernanda  Pérez Mejía </v>
+        <v>Veleria Ruiz Garcia</v>
       </c>
       <c r="C41" s="21">
         <f>+Inscritos!D39</f>
-        <v>1045143166</v>
+        <v>1038116526</v>
       </c>
       <c r="D41" s="13"/>
       <c r="E41" s="13"/>
@@ -5049,7 +5097,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I41" s="38"/>
+      <c r="I41" s="38">
+        <v>1</v>
+      </c>
       <c r="J41" s="38"/>
       <c r="K41" s="38"/>
       <c r="L41" s="38"/>
@@ -5059,7 +5109,7 @@
       <c r="P41" s="38"/>
       <c r="Q41" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R41" s="38"/>
       <c r="S41" s="38"/>
@@ -5068,7 +5118,7 @@
       <c r="V41" s="39"/>
       <c r="W41" s="39"/>
       <c r="X41" s="39"/>
-      <c r="Y41" s="38"/>
+      <c r="Y41" s="39"/>
       <c r="Z41" s="37">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -5084,15 +5134,15 @@
     </row>
     <row r="42" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A42" s="20">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B42" s="18" t="str">
         <f>+Inscritos!B40</f>
-        <v>Veleria Ruiz Garcia</v>
+        <v>Walter Antonio Perez Guzman</v>
       </c>
       <c r="C42" s="21">
         <f>+Inscritos!D40</f>
-        <v>1038116526</v>
+        <v>1040502849</v>
       </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
@@ -5102,14 +5152,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I42" s="38"/>
+      <c r="I42" s="38">
+        <v>0</v>
+      </c>
       <c r="J42" s="38"/>
       <c r="K42" s="38"/>
       <c r="L42" s="38"/>
       <c r="M42" s="38"/>
       <c r="N42" s="38"/>
       <c r="O42" s="38"/>
-      <c r="P42" s="38"/>
+      <c r="P42" s="39"/>
       <c r="Q42" s="37">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -5126,10 +5178,10 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA42" s="40"/>
-      <c r="AB42" s="39"/>
-      <c r="AC42" s="39"/>
-      <c r="AD42" s="39"/>
+      <c r="AA42" s="41"/>
+      <c r="AB42" s="42"/>
+      <c r="AC42" s="42"/>
+      <c r="AD42" s="42"/>
       <c r="AE42" s="37">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -5137,15 +5189,15 @@
     </row>
     <row r="43" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A43" s="20">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B43" s="18" t="str">
         <f>+Inscritos!B41</f>
-        <v>Walter Antonio Perez Guzman</v>
-      </c>
-      <c r="C43" s="21">
+        <v>Xiomara yiseth Causil lopez</v>
+      </c>
+      <c r="C43" s="21" t="str">
         <f>+Inscritos!D41</f>
-        <v>1040502849</v>
+        <v>1038115836</v>
       </c>
       <c r="D43" s="13"/>
       <c r="E43" s="13"/>
@@ -5155,7 +5207,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I43" s="38"/>
+      <c r="I43" s="38">
+        <v>1</v>
+      </c>
       <c r="J43" s="38"/>
       <c r="K43" s="38"/>
       <c r="L43" s="38"/>
@@ -5165,24 +5219,24 @@
       <c r="P43" s="39"/>
       <c r="Q43" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R43" s="38"/>
       <c r="S43" s="38"/>
       <c r="T43" s="38"/>
-      <c r="U43" s="39"/>
-      <c r="V43" s="39"/>
-      <c r="W43" s="39"/>
-      <c r="X43" s="39"/>
-      <c r="Y43" s="39"/>
+      <c r="U43" s="38"/>
+      <c r="V43" s="38"/>
+      <c r="W43" s="38"/>
+      <c r="X43" s="38"/>
+      <c r="Y43" s="38"/>
       <c r="Z43" s="37">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA43" s="41"/>
-      <c r="AB43" s="42"/>
-      <c r="AC43" s="42"/>
-      <c r="AD43" s="42"/>
+      <c r="AA43" s="40"/>
+      <c r="AB43" s="39"/>
+      <c r="AC43" s="39"/>
+      <c r="AD43" s="39"/>
       <c r="AE43" s="37">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -5190,15 +5244,15 @@
     </row>
     <row r="44" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A44" s="20">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B44" s="18" t="str">
         <f>+Inscritos!B42</f>
-        <v>Xiomara yiseth Causil lopez</v>
-      </c>
-      <c r="C44" s="21" t="str">
+        <v>john fredy manchego valencia</v>
+      </c>
+      <c r="C44" s="21">
         <f>+Inscritos!D42</f>
-        <v>1038115836</v>
+        <v>1038125682</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
@@ -5208,7 +5262,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I44" s="38"/>
+      <c r="I44" s="38">
+        <v>1</v>
+      </c>
       <c r="J44" s="38"/>
       <c r="K44" s="38"/>
       <c r="L44" s="38"/>
@@ -5218,7 +5274,7 @@
       <c r="P44" s="39"/>
       <c r="Q44" s="37">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="R44" s="38"/>
       <c r="S44" s="38"/>
@@ -5243,15 +5299,15 @@
     </row>
     <row r="45" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A45" s="20">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B45" s="18" t="str">
         <f>+Inscritos!B43</f>
-        <v>john fredy manchego valencia</v>
+        <v>Luz Marina Mieles Nisperuza</v>
       </c>
       <c r="C45" s="21">
         <f>+Inscritos!D43</f>
-        <v>1038125682</v>
+        <v>33104650</v>
       </c>
       <c r="D45" s="13"/>
       <c r="E45" s="13"/>
@@ -5261,7 +5317,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I45" s="38"/>
+      <c r="I45" s="38">
+        <v>0</v>
+      </c>
       <c r="J45" s="38"/>
       <c r="K45" s="38"/>
       <c r="L45" s="38"/>
@@ -5296,15 +5354,15 @@
     </row>
     <row r="46" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A46" s="20">
-        <v>41</v>
-      </c>
-      <c r="B46" s="18" t="str">
+        <v>42</v>
+      </c>
+      <c r="B46" s="18">
         <f>+Inscritos!B44</f>
-        <v>Luz Marina Mieles Nisperuza</v>
+        <v>0</v>
       </c>
       <c r="C46" s="21">
         <f>+Inscritos!D44</f>
-        <v>33104650</v>
+        <v>0</v>
       </c>
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
@@ -5321,7 +5379,7 @@
       <c r="M46" s="38"/>
       <c r="N46" s="38"/>
       <c r="O46" s="38"/>
-      <c r="P46" s="39"/>
+      <c r="P46" s="38"/>
       <c r="Q46" s="37">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -5349,7 +5407,7 @@
     </row>
     <row r="47" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A47" s="20">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B47" s="18">
         <f>+Inscritos!B45</f>
@@ -5374,7 +5432,7 @@
       <c r="M47" s="38"/>
       <c r="N47" s="38"/>
       <c r="O47" s="38"/>
-      <c r="P47" s="38"/>
+      <c r="P47" s="39"/>
       <c r="Q47" s="37">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -5402,7 +5460,7 @@
     </row>
     <row r="48" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A48" s="20">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B48" s="18">
         <f>+Inscritos!B46</f>
@@ -5455,7 +5513,7 @@
     </row>
     <row r="49" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A49" s="20">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B49" s="18">
         <f>+Inscritos!B47</f>
@@ -5508,7 +5566,7 @@
     </row>
     <row r="50" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A50" s="20">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B50" s="18">
         <f>+Inscritos!B48</f>
@@ -5533,7 +5591,7 @@
       <c r="M50" s="38"/>
       <c r="N50" s="38"/>
       <c r="O50" s="38"/>
-      <c r="P50" s="39"/>
+      <c r="P50" s="38"/>
       <c r="Q50" s="37">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -5561,7 +5619,7 @@
     </row>
     <row r="51" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A51" s="20">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B51" s="18">
         <f>+Inscritos!B49</f>
@@ -5586,7 +5644,7 @@
       <c r="M51" s="38"/>
       <c r="N51" s="38"/>
       <c r="O51" s="38"/>
-      <c r="P51" s="38"/>
+      <c r="P51" s="39"/>
       <c r="Q51" s="37">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -5614,7 +5672,7 @@
     </row>
     <row r="52" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A52" s="20">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B52" s="18">
         <f>+Inscritos!B50</f>
@@ -5667,7 +5725,7 @@
     </row>
     <row r="53" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A53" s="20">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B53" s="18">
         <f>+Inscritos!B51</f>
@@ -5709,7 +5767,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA53" s="40"/>
+      <c r="AA53" s="39"/>
       <c r="AB53" s="39"/>
       <c r="AC53" s="39"/>
       <c r="AD53" s="39"/>
@@ -5720,7 +5778,7 @@
     </row>
     <row r="54" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A54" s="20">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B54" s="18">
         <f>+Inscritos!B52</f>
@@ -5773,7 +5831,7 @@
     </row>
     <row r="55" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A55" s="20">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B55" s="18">
         <f>+Inscritos!B53</f>
@@ -5788,7 +5846,7 @@
       <c r="F55" s="13"/>
       <c r="G55" s="13"/>
       <c r="H55" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="H55:H64" si="4">+SUM(D55:G55)/4</f>
         <v>0</v>
       </c>
       <c r="I55" s="38"/>
@@ -5798,9 +5856,9 @@
       <c r="M55" s="38"/>
       <c r="N55" s="38"/>
       <c r="O55" s="38"/>
-      <c r="P55" s="39"/>
+      <c r="P55" s="38"/>
       <c r="Q55" s="37">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="Q55:Q64" si="5">+SUM(I55:P55)/8</f>
         <v>0</v>
       </c>
       <c r="R55" s="38"/>
@@ -5812,21 +5870,21 @@
       <c r="X55" s="38"/>
       <c r="Y55" s="38"/>
       <c r="Z55" s="37">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA55" s="39"/>
+        <f t="shared" ref="Z55:Z64" si="6">+SUM(R55:Y55)/8</f>
+        <v>0</v>
+      </c>
+      <c r="AA55" s="40"/>
       <c r="AB55" s="39"/>
       <c r="AC55" s="39"/>
       <c r="AD55" s="39"/>
       <c r="AE55" s="37">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="AE55:AE64" si="7">+SUM(AA55:AD55)/4</f>
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A56" s="20">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B56" s="18">
         <f>+Inscritos!B54</f>
@@ -5841,7 +5899,7 @@
       <c r="F56" s="13"/>
       <c r="G56" s="13"/>
       <c r="H56" s="37">
-        <f t="shared" ref="H56:H65" si="4">+SUM(D56:G56)/4</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I56" s="38"/>
@@ -5851,9 +5909,9 @@
       <c r="M56" s="38"/>
       <c r="N56" s="38"/>
       <c r="O56" s="38"/>
-      <c r="P56" s="38"/>
+      <c r="P56" s="39"/>
       <c r="Q56" s="37">
-        <f t="shared" ref="Q56:Q65" si="5">+SUM(I56:P56)/8</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="R56" s="38"/>
@@ -5865,7 +5923,7 @@
       <c r="X56" s="38"/>
       <c r="Y56" s="38"/>
       <c r="Z56" s="37">
-        <f t="shared" ref="Z56:Z65" si="6">+SUM(R56:Y56)/8</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AA56" s="40"/>
@@ -5873,13 +5931,13 @@
       <c r="AC56" s="39"/>
       <c r="AD56" s="39"/>
       <c r="AE56" s="37">
-        <f t="shared" ref="AE56:AE65" si="7">+SUM(AA56:AD56)/4</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A57" s="20">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B57" s="18">
         <f>+Inscritos!B55</f>
@@ -5932,7 +5990,7 @@
     </row>
     <row r="58" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A58" s="20">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B58" s="18">
         <f>+Inscritos!B56</f>
@@ -5974,7 +6032,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AA58" s="40"/>
+      <c r="AA58" s="39"/>
       <c r="AB58" s="39"/>
       <c r="AC58" s="39"/>
       <c r="AD58" s="39"/>
@@ -5985,7 +6043,7 @@
     </row>
     <row r="59" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A59" s="20">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B59" s="18">
         <f>+Inscritos!B57</f>
@@ -6038,7 +6096,7 @@
     </row>
     <row r="60" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A60" s="20">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B60" s="18">
         <f>+Inscritos!B58</f>
@@ -6063,7 +6121,7 @@
       <c r="M60" s="38"/>
       <c r="N60" s="38"/>
       <c r="O60" s="38"/>
-      <c r="P60" s="39"/>
+      <c r="P60" s="38"/>
       <c r="Q60" s="37">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -6080,7 +6138,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AA60" s="39"/>
+      <c r="AA60" s="40"/>
       <c r="AB60" s="39"/>
       <c r="AC60" s="39"/>
       <c r="AD60" s="39"/>
@@ -6091,7 +6149,7 @@
     </row>
     <row r="61" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A61" s="20">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B61" s="18">
         <f>+Inscritos!B59</f>
@@ -6116,7 +6174,7 @@
       <c r="M61" s="38"/>
       <c r="N61" s="38"/>
       <c r="O61" s="38"/>
-      <c r="P61" s="38"/>
+      <c r="P61" s="39"/>
       <c r="Q61" s="37">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -6144,7 +6202,7 @@
     </row>
     <row r="62" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A62" s="20">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B62" s="18">
         <f>+Inscritos!B60</f>
@@ -6197,7 +6255,7 @@
     </row>
     <row r="63" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A63" s="20">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B63" s="18">
         <f>+Inscritos!B61</f>
@@ -6239,7 +6297,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="AA63" s="40"/>
+      <c r="AA63" s="39"/>
       <c r="AB63" s="39"/>
       <c r="AC63" s="39"/>
       <c r="AD63" s="39"/>
@@ -6250,7 +6308,7 @@
     </row>
     <row r="64" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
       <c r="A64" s="20">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B64" s="18">
         <f>+Inscritos!B62</f>
@@ -6301,61 +6359,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:31" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A65" s="20">
-        <v>60</v>
-      </c>
-      <c r="B65" s="18">
-        <f>+Inscritos!B63</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="21">
-        <f>+Inscritos!D63</f>
-        <v>0</v>
-      </c>
-      <c r="D65" s="13"/>
-      <c r="E65" s="13"/>
-      <c r="F65" s="13"/>
-      <c r="G65" s="13"/>
-      <c r="H65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I65" s="38"/>
-      <c r="J65" s="38"/>
-      <c r="K65" s="38"/>
-      <c r="L65" s="38"/>
-      <c r="M65" s="38"/>
-      <c r="N65" s="38"/>
-      <c r="O65" s="38"/>
-      <c r="P65" s="39"/>
-      <c r="Q65" s="37">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="R65" s="38"/>
-      <c r="S65" s="38"/>
-      <c r="T65" s="38"/>
-      <c r="U65" s="38"/>
-      <c r="V65" s="38"/>
-      <c r="W65" s="38"/>
-      <c r="X65" s="38"/>
-      <c r="Y65" s="38"/>
-      <c r="Z65" s="37">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="AA65" s="39"/>
-      <c r="AB65" s="39"/>
-      <c r="AC65" s="39"/>
-      <c r="AD65" s="39"/>
-      <c r="AE65" s="37">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:H60">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:H59">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="16">
@@ -6406,30 +6411,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="86"/>
-      <c r="J1" s="86"/>
-      <c r="K1" s="86"/>
-      <c r="L1" s="86"/>
-      <c r="M1" s="86"/>
-      <c r="N1" s="86"/>
-      <c r="O1" s="86"/>
-      <c r="P1" s="86"/>
-      <c r="Q1" s="86"/>
-      <c r="R1" s="86"/>
-      <c r="S1" s="86"/>
-      <c r="T1" s="86"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="112"/>
+      <c r="T1" s="112"/>
     </row>
     <row r="2" spans="1:20" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="123" t="s">
+      <c r="A2" s="98" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="84" t="s">
@@ -6438,89 +6443,89 @@
       <c r="C2" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="114" t="str">
+      <c r="D2" s="86" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="115"/>
-      <c r="F2" s="116"/>
-      <c r="G2" s="114" t="str">
+      <c r="E2" s="87"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="86" t="str">
         <f>Asistencia!I2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="114" t="s">
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="88"/>
+      <c r="L2" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="115"/>
-      <c r="N2" s="115"/>
-      <c r="O2" s="115"/>
-      <c r="P2" s="116"/>
-      <c r="Q2" s="114" t="str">
+      <c r="M2" s="87"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="87"/>
+      <c r="P2" s="88"/>
+      <c r="Q2" s="86" t="str">
         <f>Asistencia!AA2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="115"/>
-      <c r="S2" s="115"/>
-      <c r="T2" s="116"/>
+      <c r="R2" s="87"/>
+      <c r="S2" s="87"/>
+      <c r="T2" s="88"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="124"/>
+      <c r="A3" s="99"/>
       <c r="B3" s="85"/>
       <c r="C3" s="61"/>
-      <c r="D3" s="131" t="s">
+      <c r="D3" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="132"/>
-      <c r="F3" s="133"/>
-      <c r="G3" s="125" t="s">
+      <c r="E3" s="107"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="127"/>
-      <c r="L3" s="108" t="s">
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="102"/>
+      <c r="L3" s="131" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="109"/>
-      <c r="N3" s="109"/>
-      <c r="O3" s="109"/>
-      <c r="P3" s="110"/>
-      <c r="Q3" s="117" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="118"/>
-      <c r="S3" s="118"/>
-      <c r="T3" s="119"/>
+      <c r="M3" s="132"/>
+      <c r="N3" s="132"/>
+      <c r="O3" s="132"/>
+      <c r="P3" s="133"/>
+      <c r="Q3" s="89" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="90"/>
+      <c r="S3" s="90"/>
+      <c r="T3" s="91"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="124"/>
+      <c r="A4" s="99"/>
       <c r="B4" s="85"/>
       <c r="C4" s="61"/>
-      <c r="D4" s="134"/>
-      <c r="E4" s="135"/>
-      <c r="F4" s="136"/>
-      <c r="G4" s="128"/>
-      <c r="H4" s="129"/>
-      <c r="I4" s="129"/>
-      <c r="J4" s="129"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="111"/>
-      <c r="M4" s="112"/>
-      <c r="N4" s="112"/>
-      <c r="O4" s="112"/>
-      <c r="P4" s="113"/>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="121"/>
-      <c r="S4" s="121"/>
-      <c r="T4" s="122"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="111"/>
+      <c r="G4" s="103"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="104"/>
+      <c r="J4" s="104"/>
+      <c r="K4" s="105"/>
+      <c r="L4" s="134"/>
+      <c r="M4" s="135"/>
+      <c r="N4" s="135"/>
+      <c r="O4" s="135"/>
+      <c r="P4" s="136"/>
+      <c r="Q4" s="92"/>
+      <c r="R4" s="93"/>
+      <c r="S4" s="93"/>
+      <c r="T4" s="94"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="124"/>
+      <c r="A5" s="99"/>
       <c r="B5" s="85"/>
       <c r="C5" s="61"/>
       <c r="D5" s="22">
@@ -7889,13 +7894,13 @@
       <c r="A37" s="10">
         <v>32</v>
       </c>
-      <c r="B37" s="18" t="str">
-        <f>Inscritos!B35</f>
-        <v>Sara Paulina Cardona Almanza</v>
-      </c>
-      <c r="C37" s="18">
-        <f>+Inscritos!D35</f>
-        <v>1038648764</v>
+      <c r="B37" s="18" t="e">
+        <f>Inscritos!#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C37" s="18" t="e">
+        <f>+Inscritos!#REF!</f>
+        <v>#REF!</v>
       </c>
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
@@ -7932,11 +7937,11 @@
         <v>33</v>
       </c>
       <c r="B38" s="18" t="str">
-        <f>Inscritos!B36</f>
+        <f>Inscritos!B35</f>
         <v>Sara Paulina Cardona Almanza</v>
       </c>
       <c r="C38" s="18">
-        <f>+Inscritos!D36</f>
+        <f>+Inscritos!D35</f>
         <v>1038648764</v>
       </c>
       <c r="D38" s="7"/>
@@ -7974,11 +7979,11 @@
         <v>34</v>
       </c>
       <c r="B39" s="18" t="str">
-        <f>Inscritos!B37</f>
+        <f>Inscritos!B36</f>
         <v>Sheyla Ramirez Guerra</v>
       </c>
       <c r="C39" s="18">
-        <f>+Inscritos!D37</f>
+        <f>+Inscritos!D36</f>
         <v>1038118107</v>
       </c>
       <c r="D39" s="7"/>
@@ -8016,11 +8021,11 @@
         <v>35</v>
       </c>
       <c r="B40" s="18" t="str">
-        <f>Inscritos!B38</f>
+        <f>Inscritos!B37</f>
         <v>Susana Tobon Ortega</v>
       </c>
       <c r="C40" s="18">
-        <f>+Inscritos!D38</f>
+        <f>+Inscritos!D37</f>
         <v>1020303245</v>
       </c>
       <c r="D40" s="7"/>
@@ -8058,11 +8063,11 @@
         <v>36</v>
       </c>
       <c r="B41" s="18" t="str">
-        <f>Inscritos!B39</f>
+        <f>Inscritos!B38</f>
         <v xml:space="preserve">Valerin Fernanda  Pérez Mejía </v>
       </c>
       <c r="C41" s="18">
-        <f>+Inscritos!D39</f>
+        <f>+Inscritos!D38</f>
         <v>1045143166</v>
       </c>
       <c r="D41" s="7"/>
@@ -8100,11 +8105,11 @@
         <v>37</v>
       </c>
       <c r="B42" s="18" t="str">
-        <f>Inscritos!B40</f>
+        <f>Inscritos!B39</f>
         <v>Veleria Ruiz Garcia</v>
       </c>
       <c r="C42" s="18">
-        <f>+Inscritos!D40</f>
+        <f>+Inscritos!D39</f>
         <v>1038116526</v>
       </c>
       <c r="D42" s="7"/>
@@ -8142,11 +8147,11 @@
         <v>38</v>
       </c>
       <c r="B43" s="18" t="str">
-        <f>Inscritos!B41</f>
+        <f>Inscritos!B40</f>
         <v>Walter Antonio Perez Guzman</v>
       </c>
       <c r="C43" s="18">
-        <f>+Inscritos!D41</f>
+        <f>+Inscritos!D40</f>
         <v>1040502849</v>
       </c>
       <c r="D43" s="7"/>
@@ -8184,11 +8189,11 @@
         <v>39</v>
       </c>
       <c r="B44" s="18" t="str">
-        <f>Inscritos!B42</f>
+        <f>Inscritos!B41</f>
         <v>Xiomara yiseth Causil lopez</v>
       </c>
       <c r="C44" s="18" t="str">
-        <f>+Inscritos!D42</f>
+        <f>+Inscritos!D41</f>
         <v>1038115836</v>
       </c>
       <c r="D44" s="7"/>
@@ -8226,11 +8231,11 @@
         <v>40</v>
       </c>
       <c r="B45" s="18" t="str">
-        <f>Inscritos!B43</f>
+        <f>Inscritos!B42</f>
         <v>john fredy manchego valencia</v>
       </c>
       <c r="C45" s="18">
-        <f>+Inscritos!D43</f>
+        <f>+Inscritos!D42</f>
         <v>1038125682</v>
       </c>
       <c r="D45" s="7"/>
@@ -8268,11 +8273,11 @@
         <v>41</v>
       </c>
       <c r="B46" s="18" t="str">
-        <f>Inscritos!B44</f>
+        <f>Inscritos!B43</f>
         <v>Luz Marina Mieles Nisperuza</v>
       </c>
       <c r="C46" s="18">
-        <f>+Inscritos!D44</f>
+        <f>+Inscritos!D43</f>
         <v>33104650</v>
       </c>
       <c r="D46" s="7"/>
@@ -8310,11 +8315,11 @@
         <v>42</v>
       </c>
       <c r="B47" s="18">
-        <f>Inscritos!B45</f>
+        <f>Inscritos!B44</f>
         <v>0</v>
       </c>
       <c r="C47" s="18">
-        <f>+Inscritos!D45</f>
+        <f>+Inscritos!D44</f>
         <v>0</v>
       </c>
       <c r="D47" s="7"/>
@@ -8352,11 +8357,11 @@
         <v>43</v>
       </c>
       <c r="B48" s="18">
-        <f>Inscritos!B46</f>
+        <f>Inscritos!B45</f>
         <v>0</v>
       </c>
       <c r="C48" s="18">
-        <f>+Inscritos!D46</f>
+        <f>+Inscritos!D45</f>
         <v>0</v>
       </c>
       <c r="D48" s="7"/>
@@ -8394,11 +8399,11 @@
         <v>44</v>
       </c>
       <c r="B49" s="18">
-        <f>Inscritos!B47</f>
+        <f>Inscritos!B46</f>
         <v>0</v>
       </c>
       <c r="C49" s="18">
-        <f>+Inscritos!D47</f>
+        <f>+Inscritos!D46</f>
         <v>0</v>
       </c>
       <c r="D49" s="7"/>
@@ -8436,11 +8441,11 @@
         <v>45</v>
       </c>
       <c r="B50" s="18">
-        <f>Inscritos!B48</f>
+        <f>Inscritos!B47</f>
         <v>0</v>
       </c>
       <c r="C50" s="18">
-        <f>+Inscritos!D48</f>
+        <f>+Inscritos!D47</f>
         <v>0</v>
       </c>
       <c r="D50" s="7"/>
@@ -8478,11 +8483,11 @@
         <v>46</v>
       </c>
       <c r="B51" s="18">
-        <f>Inscritos!B49</f>
+        <f>Inscritos!B48</f>
         <v>0</v>
       </c>
       <c r="C51" s="18">
-        <f>+Inscritos!D49</f>
+        <f>+Inscritos!D48</f>
         <v>0</v>
       </c>
       <c r="D51" s="7"/>
@@ -8520,11 +8525,11 @@
         <v>47</v>
       </c>
       <c r="B52" s="18">
-        <f>Inscritos!B50</f>
+        <f>Inscritos!B49</f>
         <v>0</v>
       </c>
       <c r="C52" s="18">
-        <f>+Inscritos!D50</f>
+        <f>+Inscritos!D49</f>
         <v>0</v>
       </c>
       <c r="D52" s="7"/>
@@ -8562,11 +8567,11 @@
         <v>48</v>
       </c>
       <c r="B53" s="18">
-        <f>Inscritos!B51</f>
+        <f>Inscritos!B50</f>
         <v>0</v>
       </c>
       <c r="C53" s="18">
-        <f>+Inscritos!D51</f>
+        <f>+Inscritos!D50</f>
         <v>0</v>
       </c>
       <c r="D53" s="7"/>
@@ -8604,11 +8609,11 @@
         <v>49</v>
       </c>
       <c r="B54" s="18">
-        <f>Inscritos!B52</f>
+        <f>Inscritos!B51</f>
         <v>0</v>
       </c>
       <c r="C54" s="18">
-        <f>+Inscritos!D52</f>
+        <f>+Inscritos!D51</f>
         <v>0</v>
       </c>
       <c r="D54" s="7"/>
@@ -8646,11 +8651,11 @@
         <v>50</v>
       </c>
       <c r="B55" s="18">
-        <f>Inscritos!B53</f>
+        <f>Inscritos!B52</f>
         <v>0</v>
       </c>
       <c r="C55" s="18">
-        <f>+Inscritos!D53</f>
+        <f>+Inscritos!D52</f>
         <v>0</v>
       </c>
       <c r="D55" s="7"/>
@@ -8688,11 +8693,11 @@
         <v>51</v>
       </c>
       <c r="B56" s="18">
-        <f>Inscritos!B54</f>
+        <f>Inscritos!B53</f>
         <v>0</v>
       </c>
       <c r="C56" s="18">
-        <f>+Inscritos!D54</f>
+        <f>+Inscritos!D53</f>
         <v>0</v>
       </c>
       <c r="D56" s="7"/>
@@ -8730,11 +8735,11 @@
         <v>52</v>
       </c>
       <c r="B57" s="18">
-        <f>Inscritos!B55</f>
+        <f>Inscritos!B54</f>
         <v>0</v>
       </c>
       <c r="C57" s="18">
-        <f>+Inscritos!D55</f>
+        <f>+Inscritos!D54</f>
         <v>0</v>
       </c>
       <c r="D57" s="7"/>
@@ -8772,11 +8777,11 @@
         <v>53</v>
       </c>
       <c r="B58" s="18">
-        <f>Inscritos!B56</f>
+        <f>Inscritos!B55</f>
         <v>0</v>
       </c>
       <c r="C58" s="18">
-        <f>+Inscritos!D56</f>
+        <f>+Inscritos!D55</f>
         <v>0</v>
       </c>
       <c r="D58" s="7"/>
@@ -8814,11 +8819,11 @@
         <v>54</v>
       </c>
       <c r="B59" s="18">
-        <f>Inscritos!B57</f>
+        <f>Inscritos!B56</f>
         <v>0</v>
       </c>
       <c r="C59" s="18">
-        <f>+Inscritos!D57</f>
+        <f>+Inscritos!D56</f>
         <v>0</v>
       </c>
       <c r="D59" s="7"/>
@@ -8856,11 +8861,11 @@
         <v>55</v>
       </c>
       <c r="B60" s="18">
-        <f>Inscritos!B58</f>
+        <f>Inscritos!B57</f>
         <v>0</v>
       </c>
       <c r="C60" s="18">
-        <f>+Inscritos!D58</f>
+        <f>+Inscritos!D57</f>
         <v>0</v>
       </c>
       <c r="D60" s="7"/>
@@ -8898,11 +8903,11 @@
         <v>56</v>
       </c>
       <c r="B61" s="18">
-        <f>Inscritos!B59</f>
+        <f>Inscritos!B58</f>
         <v>0</v>
       </c>
       <c r="C61" s="18">
-        <f>+Inscritos!D59</f>
+        <f>+Inscritos!D58</f>
         <v>0</v>
       </c>
       <c r="D61" s="7"/>
@@ -8940,11 +8945,11 @@
         <v>57</v>
       </c>
       <c r="B62" s="18">
-        <f>Inscritos!B60</f>
+        <f>Inscritos!B59</f>
         <v>0</v>
       </c>
       <c r="C62" s="18">
-        <f>+Inscritos!D60</f>
+        <f>+Inscritos!D59</f>
         <v>0</v>
       </c>
       <c r="D62" s="7"/>
@@ -8982,11 +8987,11 @@
         <v>58</v>
       </c>
       <c r="B63" s="18">
-        <f>Inscritos!B61</f>
+        <f>Inscritos!B60</f>
         <v>0</v>
       </c>
       <c r="C63" s="18">
-        <f>+Inscritos!D61</f>
+        <f>+Inscritos!D60</f>
         <v>0</v>
       </c>
       <c r="D63" s="7"/>
@@ -9024,11 +9029,11 @@
         <v>59</v>
       </c>
       <c r="B64" s="18">
-        <f>Inscritos!B62</f>
+        <f>Inscritos!B61</f>
         <v>0</v>
       </c>
       <c r="C64" s="18">
-        <f>+Inscritos!D62</f>
+        <f>+Inscritos!D61</f>
         <v>0</v>
       </c>
       <c r="D64" s="7"/>
@@ -9066,11 +9071,11 @@
         <v>60</v>
       </c>
       <c r="B65" s="18">
-        <f>Inscritos!B63</f>
+        <f>Inscritos!B62</f>
         <v>0</v>
       </c>
       <c r="C65" s="18">
-        <f>+Inscritos!D63</f>
+        <f>+Inscritos!D62</f>
         <v>0</v>
       </c>
       <c r="D65" s="7"/>
@@ -9104,195 +9109,186 @@
       </c>
     </row>
     <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D66" s="90" t="s">
+      <c r="D66" s="116" t="s">
         <v>26</v>
       </c>
-      <c r="E66" s="93" t="s">
+      <c r="E66" s="119" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="87" t="s">
+      <c r="G66" s="113" t="s">
         <v>8</v>
       </c>
-      <c r="H66" s="102" t="s">
+      <c r="H66" s="125" t="s">
         <v>9</v>
       </c>
-      <c r="I66" s="102" t="s">
+      <c r="I66" s="125" t="s">
         <v>10</v>
       </c>
-      <c r="J66" s="87" t="s">
+      <c r="J66" s="113" t="s">
         <v>11</v>
       </c>
-      <c r="L66" s="96" t="s">
+      <c r="L66" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="M66" s="99" t="s">
+      <c r="M66" s="122" t="s">
         <v>9</v>
       </c>
-      <c r="N66" s="99" t="s">
+      <c r="N66" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="O66" s="96" t="s">
+      <c r="O66" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="Q66" s="105" t="s">
+      <c r="Q66" s="128" t="s">
         <v>26</v>
       </c>
-      <c r="R66" s="105" t="s">
+      <c r="R66" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="S66" s="105" t="s">
+      <c r="S66" s="128" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D67" s="91"/>
-      <c r="E67" s="94"/>
-      <c r="G67" s="88"/>
-      <c r="H67" s="103"/>
-      <c r="I67" s="103"/>
-      <c r="J67" s="88"/>
-      <c r="L67" s="97"/>
-      <c r="M67" s="100"/>
-      <c r="N67" s="100"/>
-      <c r="O67" s="97"/>
-      <c r="Q67" s="106"/>
-      <c r="R67" s="106"/>
-      <c r="S67" s="106"/>
+      <c r="D67" s="117"/>
+      <c r="E67" s="120"/>
+      <c r="G67" s="114"/>
+      <c r="H67" s="126"/>
+      <c r="I67" s="126"/>
+      <c r="J67" s="114"/>
+      <c r="L67" s="96"/>
+      <c r="M67" s="123"/>
+      <c r="N67" s="123"/>
+      <c r="O67" s="96"/>
+      <c r="Q67" s="129"/>
+      <c r="R67" s="129"/>
+      <c r="S67" s="129"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D68" s="91"/>
-      <c r="E68" s="94"/>
-      <c r="G68" s="88"/>
-      <c r="H68" s="103"/>
-      <c r="I68" s="103"/>
-      <c r="J68" s="88"/>
-      <c r="L68" s="97"/>
-      <c r="M68" s="100"/>
-      <c r="N68" s="100"/>
-      <c r="O68" s="97"/>
-      <c r="Q68" s="106"/>
-      <c r="R68" s="106"/>
-      <c r="S68" s="106"/>
+      <c r="D68" s="117"/>
+      <c r="E68" s="120"/>
+      <c r="G68" s="114"/>
+      <c r="H68" s="126"/>
+      <c r="I68" s="126"/>
+      <c r="J68" s="114"/>
+      <c r="L68" s="96"/>
+      <c r="M68" s="123"/>
+      <c r="N68" s="123"/>
+      <c r="O68" s="96"/>
+      <c r="Q68" s="129"/>
+      <c r="R68" s="129"/>
+      <c r="S68" s="129"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D69" s="91"/>
-      <c r="E69" s="94"/>
-      <c r="G69" s="88"/>
-      <c r="H69" s="103"/>
-      <c r="I69" s="103"/>
-      <c r="J69" s="88"/>
-      <c r="L69" s="97"/>
-      <c r="M69" s="100"/>
-      <c r="N69" s="100"/>
-      <c r="O69" s="97"/>
-      <c r="Q69" s="106"/>
-      <c r="R69" s="106"/>
-      <c r="S69" s="106"/>
+      <c r="D69" s="117"/>
+      <c r="E69" s="120"/>
+      <c r="G69" s="114"/>
+      <c r="H69" s="126"/>
+      <c r="I69" s="126"/>
+      <c r="J69" s="114"/>
+      <c r="L69" s="96"/>
+      <c r="M69" s="123"/>
+      <c r="N69" s="123"/>
+      <c r="O69" s="96"/>
+      <c r="Q69" s="129"/>
+      <c r="R69" s="129"/>
+      <c r="S69" s="129"/>
     </row>
     <row r="70" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D70" s="91"/>
-      <c r="E70" s="94"/>
-      <c r="G70" s="88"/>
-      <c r="H70" s="103"/>
-      <c r="I70" s="103"/>
-      <c r="J70" s="88"/>
-      <c r="L70" s="97"/>
-      <c r="M70" s="100"/>
-      <c r="N70" s="100"/>
-      <c r="O70" s="97"/>
-      <c r="Q70" s="106"/>
-      <c r="R70" s="106"/>
-      <c r="S70" s="106"/>
+      <c r="D70" s="117"/>
+      <c r="E70" s="120"/>
+      <c r="G70" s="114"/>
+      <c r="H70" s="126"/>
+      <c r="I70" s="126"/>
+      <c r="J70" s="114"/>
+      <c r="L70" s="96"/>
+      <c r="M70" s="123"/>
+      <c r="N70" s="123"/>
+      <c r="O70" s="96"/>
+      <c r="Q70" s="129"/>
+      <c r="R70" s="129"/>
+      <c r="S70" s="129"/>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D71" s="91"/>
-      <c r="E71" s="94"/>
-      <c r="G71" s="88"/>
-      <c r="H71" s="103"/>
-      <c r="I71" s="103"/>
-      <c r="J71" s="88"/>
-      <c r="L71" s="97"/>
-      <c r="M71" s="100"/>
-      <c r="N71" s="100"/>
-      <c r="O71" s="97"/>
-      <c r="Q71" s="106"/>
-      <c r="R71" s="106"/>
-      <c r="S71" s="106"/>
+      <c r="D71" s="117"/>
+      <c r="E71" s="120"/>
+      <c r="G71" s="114"/>
+      <c r="H71" s="126"/>
+      <c r="I71" s="126"/>
+      <c r="J71" s="114"/>
+      <c r="L71" s="96"/>
+      <c r="M71" s="123"/>
+      <c r="N71" s="123"/>
+      <c r="O71" s="96"/>
+      <c r="Q71" s="129"/>
+      <c r="R71" s="129"/>
+      <c r="S71" s="129"/>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D72" s="91"/>
-      <c r="E72" s="94"/>
-      <c r="G72" s="88"/>
-      <c r="H72" s="103"/>
-      <c r="I72" s="103"/>
-      <c r="J72" s="88"/>
-      <c r="L72" s="97"/>
-      <c r="M72" s="100"/>
-      <c r="N72" s="100"/>
-      <c r="O72" s="97"/>
-      <c r="Q72" s="106"/>
-      <c r="R72" s="106"/>
-      <c r="S72" s="106"/>
+      <c r="D72" s="117"/>
+      <c r="E72" s="120"/>
+      <c r="G72" s="114"/>
+      <c r="H72" s="126"/>
+      <c r="I72" s="126"/>
+      <c r="J72" s="114"/>
+      <c r="L72" s="96"/>
+      <c r="M72" s="123"/>
+      <c r="N72" s="123"/>
+      <c r="O72" s="96"/>
+      <c r="Q72" s="129"/>
+      <c r="R72" s="129"/>
+      <c r="S72" s="129"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D73" s="91"/>
-      <c r="E73" s="94"/>
-      <c r="G73" s="88"/>
-      <c r="H73" s="103"/>
-      <c r="I73" s="103"/>
-      <c r="J73" s="88"/>
-      <c r="L73" s="97"/>
-      <c r="M73" s="100"/>
-      <c r="N73" s="100"/>
-      <c r="O73" s="97"/>
-      <c r="Q73" s="106"/>
-      <c r="R73" s="106"/>
-      <c r="S73" s="106"/>
+      <c r="D73" s="117"/>
+      <c r="E73" s="120"/>
+      <c r="G73" s="114"/>
+      <c r="H73" s="126"/>
+      <c r="I73" s="126"/>
+      <c r="J73" s="114"/>
+      <c r="L73" s="96"/>
+      <c r="M73" s="123"/>
+      <c r="N73" s="123"/>
+      <c r="O73" s="96"/>
+      <c r="Q73" s="129"/>
+      <c r="R73" s="129"/>
+      <c r="S73" s="129"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="D74" s="91"/>
-      <c r="E74" s="94"/>
-      <c r="G74" s="88"/>
-      <c r="H74" s="103"/>
-      <c r="I74" s="103"/>
-      <c r="J74" s="88"/>
-      <c r="L74" s="97"/>
-      <c r="M74" s="100"/>
-      <c r="N74" s="100"/>
-      <c r="O74" s="97"/>
-      <c r="Q74" s="106"/>
-      <c r="R74" s="106"/>
-      <c r="S74" s="106"/>
+      <c r="D74" s="117"/>
+      <c r="E74" s="120"/>
+      <c r="G74" s="114"/>
+      <c r="H74" s="126"/>
+      <c r="I74" s="126"/>
+      <c r="J74" s="114"/>
+      <c r="L74" s="96"/>
+      <c r="M74" s="123"/>
+      <c r="N74" s="123"/>
+      <c r="O74" s="96"/>
+      <c r="Q74" s="129"/>
+      <c r="R74" s="129"/>
+      <c r="S74" s="129"/>
     </row>
     <row r="75" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D75" s="92"/>
-      <c r="E75" s="95"/>
-      <c r="G75" s="89"/>
-      <c r="H75" s="104"/>
-      <c r="I75" s="104"/>
-      <c r="J75" s="89"/>
-      <c r="L75" s="98"/>
-      <c r="M75" s="101"/>
-      <c r="N75" s="101"/>
-      <c r="O75" s="98"/>
-      <c r="Q75" s="107"/>
-      <c r="R75" s="107"/>
-      <c r="S75" s="107"/>
+      <c r="D75" s="118"/>
+      <c r="E75" s="121"/>
+      <c r="G75" s="115"/>
+      <c r="H75" s="127"/>
+      <c r="I75" s="127"/>
+      <c r="J75" s="115"/>
+      <c r="L75" s="97"/>
+      <c r="M75" s="124"/>
+      <c r="N75" s="124"/>
+      <c r="O75" s="97"/>
+      <c r="Q75" s="130"/>
+      <c r="R75" s="130"/>
+      <c r="S75" s="130"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:T60">
     <sortCondition ref="B6"/>
   </sortState>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O66:O75"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J66:J75"/>
     <mergeCell ref="D66:D75"/>
@@ -9309,6 +9305,15 @@
     <mergeCell ref="I66:I75"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O66:O75"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>